<commit_message>
#3 (Cost Optimization for 5 and 1000 pcs)
</commit_message>
<xml_diff>
--- a/Design Files/LLR-05U (Advance Version)/Secondary Board/BOM/eSpark BOM LLR-05U (Secondary-Board).xlsx
+++ b/Design Files/LLR-05U (Advance Version)/Secondary Board/BOM/eSpark BOM LLR-05U (Secondary-Board).xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\abdullah-liquidlevelrelay\Design Files\LLR-05U (Advance Version)\Secondary Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6850ED96-564E-4B00-AAC6-9F5B9A3E21C0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAE00AFA-0E5E-4294-9649-F4D88036687F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
     <sheet name="1000 Boards" sheetId="2" r:id="rId2"/>
     <sheet name="5 Boards Low Cost" sheetId="3" r:id="rId3"/>
+    <sheet name="1000 Boards Low Cost" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="137">
   <si>
     <t>Component list</t>
   </si>
@@ -1140,6 +1141,60 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1752600</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>84833</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{59CF3857-C0AF-4A5D-B314-0B9FDF8B5842}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25812750" y="257175"/>
+          <a:ext cx="1714500" cy="1361183"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4263,12 +4318,18 @@
         <f>L12*5</f>
         <v>5</v>
       </c>
-      <c r="N12" s="43"/>
-      <c r="O12" s="45"/>
-      <c r="P12" s="47"/>
+      <c r="N12" s="43">
+        <v>100</v>
+      </c>
+      <c r="O12" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P12" s="47">
+        <v>6.0000000000000001E-3</v>
+      </c>
       <c r="Q12" s="15">
         <f>P12*N12</f>
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="R12" s="14"/>
       <c r="S12" s="20"/>
@@ -4311,12 +4372,18 @@
         <f t="shared" ref="M13" si="5">L13*5</f>
         <v>15</v>
       </c>
-      <c r="N13" s="44"/>
-      <c r="O13" s="46"/>
-      <c r="P13" s="48"/>
+      <c r="N13" s="44">
+        <v>100</v>
+      </c>
+      <c r="O13" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P13" s="48">
+        <v>4.4999999999999997E-3</v>
+      </c>
       <c r="Q13" s="22">
         <f t="shared" ref="Q13" si="6">P13*N13</f>
-        <v>0</v>
+        <v>0.44999999999999996</v>
       </c>
       <c r="R13" s="21"/>
       <c r="S13" s="21"/>
@@ -4407,12 +4474,18 @@
         <f t="shared" ref="M15" si="7">L15*5</f>
         <v>15</v>
       </c>
-      <c r="N15" s="44"/>
-      <c r="O15" s="46"/>
-      <c r="P15" s="48"/>
+      <c r="N15" s="44">
+        <v>100</v>
+      </c>
+      <c r="O15" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P15" s="48">
+        <v>7.1999999999999998E-3</v>
+      </c>
       <c r="Q15" s="22">
         <f t="shared" ref="Q15" si="8">P15*N15</f>
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="R15" s="21"/>
       <c r="S15" s="21"/>
@@ -4455,12 +4528,18 @@
         <f>L16*5</f>
         <v>5</v>
       </c>
-      <c r="N16" s="43"/>
-      <c r="O16" s="45"/>
-      <c r="P16" s="47"/>
+      <c r="N16" s="43">
+        <v>10</v>
+      </c>
+      <c r="O16" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P16" s="47">
+        <v>1.5100000000000001E-2</v>
+      </c>
       <c r="Q16" s="15">
         <f>P16*N16</f>
-        <v>0</v>
+        <v>0.151</v>
       </c>
       <c r="R16" s="14"/>
       <c r="S16" s="20"/>
@@ -4503,12 +4582,18 @@
         <f t="shared" ref="M17" si="9">L17*5</f>
         <v>35</v>
       </c>
-      <c r="N17" s="44"/>
-      <c r="O17" s="46"/>
-      <c r="P17" s="48"/>
+      <c r="N17" s="44">
+        <v>100</v>
+      </c>
+      <c r="O17" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P17" s="48">
+        <v>6.9999999999999999E-4</v>
+      </c>
       <c r="Q17" s="22">
         <f t="shared" ref="Q17" si="10">P17*N17</f>
-        <v>0</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="R17" s="21"/>
       <c r="S17" s="21"/>
@@ -4551,12 +4636,18 @@
         <f>L18*5</f>
         <v>20</v>
       </c>
-      <c r="N18" s="43"/>
-      <c r="O18" s="45"/>
-      <c r="P18" s="47"/>
+      <c r="N18" s="43">
+        <v>100</v>
+      </c>
+      <c r="O18" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P18" s="47">
+        <v>6.9999999999999999E-4</v>
+      </c>
       <c r="Q18" s="15">
         <f>P18*N18</f>
-        <v>0</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="R18" s="14"/>
       <c r="S18" s="20"/>
@@ -4599,12 +4690,18 @@
         <f t="shared" ref="M19" si="11">L19*5</f>
         <v>15</v>
       </c>
-      <c r="N19" s="44"/>
-      <c r="O19" s="46"/>
-      <c r="P19" s="48"/>
+      <c r="N19" s="44">
+        <v>100</v>
+      </c>
+      <c r="O19" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P19" s="48">
+        <v>6.9999999999999999E-4</v>
+      </c>
       <c r="Q19" s="22">
         <f t="shared" ref="Q19" si="12">P19*N19</f>
-        <v>0</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="R19" s="21"/>
       <c r="S19" s="21"/>
@@ -4647,12 +4744,18 @@
         <f>L20*5</f>
         <v>15</v>
       </c>
-      <c r="N20" s="43"/>
-      <c r="O20" s="45"/>
-      <c r="P20" s="47"/>
+      <c r="N20" s="43">
+        <v>100</v>
+      </c>
+      <c r="O20" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P20" s="47">
+        <v>5.0000000000000001E-4</v>
+      </c>
       <c r="Q20" s="15">
         <f>P20*N20</f>
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="R20" s="14"/>
       <c r="S20" s="20"/>
@@ -4695,12 +4798,18 @@
         <f t="shared" ref="M21" si="13">L21*5</f>
         <v>15</v>
       </c>
-      <c r="N21" s="44"/>
-      <c r="O21" s="46"/>
-      <c r="P21" s="48"/>
+      <c r="N21" s="44">
+        <v>100</v>
+      </c>
+      <c r="O21" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P21" s="48">
+        <v>4.0000000000000002E-4</v>
+      </c>
       <c r="Q21" s="22">
         <f t="shared" ref="Q21" si="14">P21*N21</f>
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="R21" s="21"/>
       <c r="S21" s="21"/>
@@ -4743,12 +4852,18 @@
         <f>L22*5</f>
         <v>5</v>
       </c>
-      <c r="N22" s="43"/>
-      <c r="O22" s="45"/>
-      <c r="P22" s="47"/>
+      <c r="N22" s="43">
+        <v>100</v>
+      </c>
+      <c r="O22" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P22" s="47">
+        <v>1.9E-3</v>
+      </c>
       <c r="Q22" s="15">
         <f>P22*N22</f>
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="R22" s="14"/>
       <c r="S22" s="20"/>
@@ -4789,12 +4904,18 @@
         <f t="shared" ref="M23" si="15">L23*5</f>
         <v>5</v>
       </c>
-      <c r="N23" s="44"/>
-      <c r="O23" s="46"/>
-      <c r="P23" s="48"/>
+      <c r="N23" s="44">
+        <v>5</v>
+      </c>
+      <c r="O23" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P23" s="48">
+        <v>1.2563</v>
+      </c>
       <c r="Q23" s="22">
         <f t="shared" ref="Q23" si="16">P23*N23</f>
-        <v>0</v>
+        <v>6.2814999999999994</v>
       </c>
       <c r="R23" s="21"/>
       <c r="S23" s="21"/>
@@ -4837,12 +4958,18 @@
         <f>L24*5</f>
         <v>5</v>
       </c>
-      <c r="N24" s="43"/>
-      <c r="O24" s="45"/>
-      <c r="P24" s="47"/>
+      <c r="N24" s="43">
+        <v>20</v>
+      </c>
+      <c r="O24" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P24" s="47">
+        <v>1.44E-2</v>
+      </c>
       <c r="Q24" s="15">
         <f>P24*N24</f>
-        <v>0</v>
+        <v>0.28799999999999998</v>
       </c>
       <c r="R24" s="14"/>
       <c r="S24" s="20"/>
@@ -4868,7 +4995,7 @@
       <c r="P25" s="52"/>
       <c r="Q25" s="18">
         <f>SUM(Q8:Q24)</f>
-        <v>1.1200000000000001</v>
+        <v>10.100499999999998</v>
       </c>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
@@ -4894,7 +5021,7 @@
       <c r="P26" s="52"/>
       <c r="Q26" s="19">
         <f>Q25/5</f>
-        <v>0.22400000000000003</v>
+        <v>2.0200999999999998</v>
       </c>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
@@ -4913,9 +5040,1219 @@
     <hyperlink ref="O8" r:id="rId1" xr:uid="{BA3F299B-A3CE-4349-AEF9-C4022D11D654}"/>
     <hyperlink ref="O9" r:id="rId2" xr:uid="{67A7F3FB-1AC8-45ED-BE3E-16E244636D00}"/>
     <hyperlink ref="O10" r:id="rId3" xr:uid="{A83FBDAD-6A51-4946-87D6-534FFEBD7ADE}"/>
+    <hyperlink ref="O12" r:id="rId4" xr:uid="{B1AC01F7-EFC1-458E-8698-65A5FFC3D5D4}"/>
+    <hyperlink ref="O13" r:id="rId5" xr:uid="{8F4DA70A-FC62-44A7-99FA-ADE8EEAB98B6}"/>
+    <hyperlink ref="O15" r:id="rId6" xr:uid="{5E8841C3-009E-491B-8175-90993618DDCF}"/>
+    <hyperlink ref="O16" r:id="rId7" xr:uid="{1DACC053-5FDD-4770-9165-5CC65BEF68AB}"/>
+    <hyperlink ref="O17" r:id="rId8" xr:uid="{5463C1AC-EF11-404D-A933-66AAC05F61CA}"/>
+    <hyperlink ref="O18" r:id="rId9" xr:uid="{1F799ADB-5F1B-4795-A0E2-AA10DDEFA4FF}"/>
+    <hyperlink ref="O19" r:id="rId10" xr:uid="{53A92BDA-018D-4A96-8A27-F5B1D9B38693}"/>
+    <hyperlink ref="O20" r:id="rId11" xr:uid="{6491F951-971D-4C6F-970D-CBDA258D86FD}"/>
+    <hyperlink ref="O21" r:id="rId12" xr:uid="{3AA63DEA-B21A-4F9F-8A31-6A3211F1CC8E}"/>
+    <hyperlink ref="O22" r:id="rId13" xr:uid="{7E8EEF43-AB22-49DB-8C88-D4CAF04B819B}"/>
+    <hyperlink ref="O23" r:id="rId14" xr:uid="{23B72340-7062-40CF-9C96-CF19052BAC73}"/>
+    <hyperlink ref="O24" r:id="rId15" xr:uid="{DBDD888A-19E2-4C45-90AC-B3726FABBC25}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
-  <drawing r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId16"/>
+  <drawing r:id="rId17"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40B2B900-C6F9-489B-AF3F-CC16D37B5992}">
+  <dimension ref="A1:S38"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="3.140625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="18" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.42578125" customWidth="1"/>
+    <col min="5" max="5" width="30.85546875" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="49"/>
+      <c r="L1" s="49"/>
+      <c r="M1" s="49"/>
+      <c r="N1" s="49"/>
+      <c r="O1" s="49"/>
+      <c r="P1" s="49"/>
+      <c r="Q1" s="49"/>
+      <c r="R1" s="49"/>
+      <c r="S1" s="50"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1">
+      <c r="A2" s="1"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="41" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="33"/>
+      <c r="Q2" s="33"/>
+      <c r="R2" s="33"/>
+      <c r="S2" s="53"/>
+    </row>
+    <row r="3" spans="1:19" ht="16.5" thickBot="1">
+      <c r="A3" s="1"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="28"/>
+      <c r="F3" s="42" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="30"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="25"/>
+      <c r="N3" s="25"/>
+      <c r="O3" s="25"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="25"/>
+      <c r="R3" s="25"/>
+      <c r="S3" s="54"/>
+    </row>
+    <row r="4" spans="1:19">
+      <c r="A4" s="1"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
+      <c r="N4" s="25"/>
+      <c r="O4" s="25"/>
+      <c r="P4" s="25"/>
+      <c r="Q4" s="25"/>
+      <c r="R4" s="25"/>
+      <c r="S4" s="54"/>
+    </row>
+    <row r="5" spans="1:19">
+      <c r="A5" s="1"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="36"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="36"/>
+      <c r="N5" s="36"/>
+      <c r="O5" s="36"/>
+      <c r="P5" s="36"/>
+      <c r="Q5" s="36"/>
+      <c r="R5" s="36"/>
+      <c r="S5" s="54"/>
+    </row>
+    <row r="6" spans="1:19" ht="15.75" thickBot="1">
+      <c r="A6" s="1"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="36"/>
+      <c r="I6" s="35"/>
+      <c r="J6" s="36"/>
+      <c r="K6" s="36"/>
+      <c r="L6" s="36"/>
+      <c r="M6" s="36"/>
+      <c r="N6" s="36"/>
+      <c r="O6" s="36"/>
+      <c r="P6" s="36"/>
+      <c r="Q6" s="36"/>
+      <c r="R6" s="36"/>
+      <c r="S6" s="55"/>
+    </row>
+    <row r="7" spans="1:19" ht="15.75" thickBot="1">
+      <c r="A7" s="1"/>
+      <c r="B7" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="L7" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="M7" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="N7" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="O7" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="P7" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="Q7" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="R7" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="S7" s="12" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="36">
+      <c r="A8" s="1"/>
+      <c r="B8" s="16">
+        <f>ROW(B8) - ROW($B$7)</f>
+        <v>1</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="L8" s="14">
+        <v>1</v>
+      </c>
+      <c r="M8" s="14">
+        <f>L8*1000</f>
+        <v>1000</v>
+      </c>
+      <c r="N8" s="43">
+        <v>1000</v>
+      </c>
+      <c r="O8" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P8" s="47">
+        <v>1.44E-2</v>
+      </c>
+      <c r="Q8" s="15">
+        <f>P8*N8</f>
+        <v>14.4</v>
+      </c>
+      <c r="R8" s="14"/>
+      <c r="S8" s="20"/>
+    </row>
+    <row r="9" spans="1:19">
+      <c r="A9" s="1"/>
+      <c r="B9" s="17">
+        <f t="shared" ref="B9:B23" si="0">ROW(B9) - ROW($B$7)</f>
+        <v>2</v>
+      </c>
+      <c r="C9" s="24"/>
+      <c r="D9" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="K9" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="L9" s="21">
+        <v>2</v>
+      </c>
+      <c r="M9" s="14">
+        <f t="shared" ref="M9:M24" si="1">L9*1000</f>
+        <v>2000</v>
+      </c>
+      <c r="N9" s="44">
+        <v>2000</v>
+      </c>
+      <c r="O9" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P9" s="48">
+        <v>3.5000000000000001E-3</v>
+      </c>
+      <c r="Q9" s="22">
+        <f t="shared" ref="Q9" si="2">P9*N9</f>
+        <v>7</v>
+      </c>
+      <c r="R9" s="21"/>
+      <c r="S9" s="21"/>
+    </row>
+    <row r="10" spans="1:19">
+      <c r="A10" s="1"/>
+      <c r="B10" s="16">
+        <f>ROW(B10) - ROW($B$7)</f>
+        <v>3</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="L10" s="14">
+        <v>3</v>
+      </c>
+      <c r="M10" s="14">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
+      <c r="N10" s="43">
+        <v>3000</v>
+      </c>
+      <c r="O10" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P10" s="47">
+        <v>2.3999999999999998E-3</v>
+      </c>
+      <c r="Q10" s="15">
+        <f>P10*N10</f>
+        <v>7.1999999999999993</v>
+      </c>
+      <c r="R10" s="14"/>
+      <c r="S10" s="20"/>
+    </row>
+    <row r="11" spans="1:19" ht="60">
+      <c r="A11" s="1"/>
+      <c r="B11" s="17">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="I11" s="21"/>
+      <c r="J11" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="K11" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="L11" s="21">
+        <v>1</v>
+      </c>
+      <c r="M11" s="14">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N11" s="44"/>
+      <c r="O11" s="46"/>
+      <c r="P11" s="48"/>
+      <c r="Q11" s="22">
+        <f t="shared" ref="Q11" si="3">P11*N11</f>
+        <v>0</v>
+      </c>
+      <c r="R11" s="21"/>
+      <c r="S11" s="21"/>
+    </row>
+    <row r="12" spans="1:19" ht="24">
+      <c r="A12" s="1"/>
+      <c r="B12" s="16">
+        <f>ROW(B12) - ROW($B$7)</f>
+        <v>5</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="K12" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="L12" s="14">
+        <v>1</v>
+      </c>
+      <c r="M12" s="14">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N12" s="43">
+        <v>1000</v>
+      </c>
+      <c r="O12" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P12" s="47">
+        <v>4.7999999999999996E-3</v>
+      </c>
+      <c r="Q12" s="15">
+        <f>P12*N12</f>
+        <v>4.8</v>
+      </c>
+      <c r="R12" s="14"/>
+      <c r="S12" s="20"/>
+    </row>
+    <row r="13" spans="1:19" ht="48">
+      <c r="A13" s="1"/>
+      <c r="B13" s="17">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="I13" s="21"/>
+      <c r="J13" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="K13" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="L13" s="21">
+        <v>3</v>
+      </c>
+      <c r="M13" s="14">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
+      <c r="N13" s="44">
+        <v>3000</v>
+      </c>
+      <c r="O13" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P13" s="48">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="Q13" s="22">
+        <f t="shared" ref="Q13" si="4">P13*N13</f>
+        <v>9.2999999999999989</v>
+      </c>
+      <c r="R13" s="21"/>
+      <c r="S13" s="21"/>
+    </row>
+    <row r="14" spans="1:19">
+      <c r="A14" s="1"/>
+      <c r="B14" s="16">
+        <f>ROW(B14) - ROW($B$7)</f>
+        <v>7</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="I14" s="14"/>
+      <c r="J14" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="K14" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="L14" s="14">
+        <v>2</v>
+      </c>
+      <c r="M14" s="14">
+        <f t="shared" si="1"/>
+        <v>2000</v>
+      </c>
+      <c r="N14" s="43"/>
+      <c r="O14" s="43"/>
+      <c r="P14" s="47"/>
+      <c r="Q14" s="15">
+        <f>P14*N14</f>
+        <v>0</v>
+      </c>
+      <c r="R14" s="14"/>
+      <c r="S14" s="20"/>
+    </row>
+    <row r="15" spans="1:19" ht="24">
+      <c r="A15" s="1"/>
+      <c r="B15" s="17">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="H15" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" s="21"/>
+      <c r="J15" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="K15" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="L15" s="21">
+        <v>3</v>
+      </c>
+      <c r="M15" s="14">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
+      <c r="N15" s="44">
+        <v>3000</v>
+      </c>
+      <c r="O15" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P15" s="48">
+        <v>4.5999999999999999E-3</v>
+      </c>
+      <c r="Q15" s="22">
+        <f t="shared" ref="Q15" si="5">P15*N15</f>
+        <v>13.799999999999999</v>
+      </c>
+      <c r="R15" s="21"/>
+      <c r="S15" s="21"/>
+    </row>
+    <row r="16" spans="1:19" ht="36">
+      <c r="A16" s="1"/>
+      <c r="B16" s="16">
+        <f>ROW(B16) - ROW($B$7)</f>
+        <v>9</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="L16" s="14">
+        <v>1</v>
+      </c>
+      <c r="M16" s="14">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N16" s="43">
+        <v>1000</v>
+      </c>
+      <c r="O16" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P16" s="47">
+        <v>1.2E-2</v>
+      </c>
+      <c r="Q16" s="15">
+        <f>P16*N16</f>
+        <v>12</v>
+      </c>
+      <c r="R16" s="14"/>
+      <c r="S16" s="20"/>
+    </row>
+    <row r="17" spans="1:19">
+      <c r="A17" s="1"/>
+      <c r="B17" s="17">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="G17" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="I17" s="21"/>
+      <c r="J17" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="K17" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="L17" s="21">
+        <v>7</v>
+      </c>
+      <c r="M17" s="14">
+        <f t="shared" si="1"/>
+        <v>7000</v>
+      </c>
+      <c r="N17" s="44">
+        <v>7000</v>
+      </c>
+      <c r="O17" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P17" s="48">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="Q17" s="22">
+        <f t="shared" ref="Q17" si="6">P17*N17</f>
+        <v>3.5</v>
+      </c>
+      <c r="R17" s="21"/>
+      <c r="S17" s="21"/>
+    </row>
+    <row r="18" spans="1:19">
+      <c r="A18" s="1"/>
+      <c r="B18" s="16">
+        <f>ROW(B18) - ROW($B$7)</f>
+        <v>11</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="K18" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="L18" s="14">
+        <v>4</v>
+      </c>
+      <c r="M18" s="14">
+        <f t="shared" si="1"/>
+        <v>4000</v>
+      </c>
+      <c r="N18" s="43">
+        <v>4000</v>
+      </c>
+      <c r="O18" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P18" s="47">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="Q18" s="15">
+        <f>P18*N18</f>
+        <v>2.4</v>
+      </c>
+      <c r="R18" s="14"/>
+      <c r="S18" s="20"/>
+    </row>
+    <row r="19" spans="1:19">
+      <c r="A19" s="1"/>
+      <c r="B19" s="17">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="G19" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="H19" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="I19" s="21"/>
+      <c r="J19" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="K19" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="L19" s="21">
+        <v>3</v>
+      </c>
+      <c r="M19" s="14">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
+      <c r="N19" s="44">
+        <v>3000</v>
+      </c>
+      <c r="O19" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P19" s="48">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="Q19" s="22">
+        <f t="shared" ref="Q19" si="7">P19*N19</f>
+        <v>1.7999999999999998</v>
+      </c>
+      <c r="R19" s="21"/>
+      <c r="S19" s="21"/>
+    </row>
+    <row r="20" spans="1:19" ht="36">
+      <c r="A20" s="1"/>
+      <c r="B20" s="16">
+        <f>ROW(B20) - ROW($B$7)</f>
+        <v>13</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="H20" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="K20" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="L20" s="14">
+        <v>3</v>
+      </c>
+      <c r="M20" s="14">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
+      <c r="N20" s="43">
+        <v>3000</v>
+      </c>
+      <c r="O20" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P20" s="47">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="Q20" s="15">
+        <f>P20*N20</f>
+        <v>1.5</v>
+      </c>
+      <c r="R20" s="14"/>
+      <c r="S20" s="20"/>
+    </row>
+    <row r="21" spans="1:19">
+      <c r="A21" s="1"/>
+      <c r="B21" s="17">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="H21" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="I21" s="21"/>
+      <c r="J21" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="K21" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="L21" s="21">
+        <v>3</v>
+      </c>
+      <c r="M21" s="14">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
+      <c r="N21" s="44">
+        <v>3000</v>
+      </c>
+      <c r="O21" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P21" s="48">
+        <v>4.0000000000000002E-4</v>
+      </c>
+      <c r="Q21" s="22">
+        <f t="shared" ref="Q21" si="8">P21*N21</f>
+        <v>1.2</v>
+      </c>
+      <c r="R21" s="21"/>
+      <c r="S21" s="21"/>
+    </row>
+    <row r="22" spans="1:19" ht="36">
+      <c r="A22" s="1"/>
+      <c r="B22" s="16">
+        <f>ROW(B22) - ROW($B$7)</f>
+        <v>15</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="H22" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="K22" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="L22" s="14">
+        <v>1</v>
+      </c>
+      <c r="M22" s="14">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N22" s="43">
+        <v>1000</v>
+      </c>
+      <c r="O22" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P22" s="47">
+        <v>1.5E-3</v>
+      </c>
+      <c r="Q22" s="15">
+        <f>P22*N22</f>
+        <v>1.5</v>
+      </c>
+      <c r="R22" s="14"/>
+      <c r="S22" s="20"/>
+    </row>
+    <row r="23" spans="1:19">
+      <c r="A23" s="1"/>
+      <c r="B23" s="17">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="E23" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="F23" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="G23" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="H23" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="L23" s="21">
+        <v>1</v>
+      </c>
+      <c r="M23" s="14">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N23" s="44">
+        <v>1000</v>
+      </c>
+      <c r="O23" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="P23" s="48">
+        <v>0.75049999999999994</v>
+      </c>
+      <c r="Q23" s="22">
+        <f t="shared" ref="Q23" si="9">P23*N23</f>
+        <v>750.5</v>
+      </c>
+      <c r="R23" s="21"/>
+      <c r="S23" s="21"/>
+    </row>
+    <row r="24" spans="1:19" ht="15.75" thickBot="1">
+      <c r="A24" s="1"/>
+      <c r="B24" s="16">
+        <f>ROW(B24) - ROW($B$7)</f>
+        <v>17</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="G24" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="K24" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="L24" s="14">
+        <v>1</v>
+      </c>
+      <c r="M24" s="14">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="N24" s="43">
+        <v>1000</v>
+      </c>
+      <c r="O24" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="P24" s="47">
+        <v>1.3899999999999999E-2</v>
+      </c>
+      <c r="Q24" s="15">
+        <f>P24*N24</f>
+        <v>13.899999999999999</v>
+      </c>
+      <c r="R24" s="14"/>
+      <c r="S24" s="20"/>
+    </row>
+    <row r="25" spans="1:19" ht="19.5" thickBot="1">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="O25" s="52"/>
+      <c r="P25" s="52"/>
+      <c r="Q25" s="18">
+        <f>SUM(Q8:Q24)</f>
+        <v>844.8</v>
+      </c>
+      <c r="R25" s="1"/>
+      <c r="S25" s="1"/>
+    </row>
+    <row r="26" spans="1:19" ht="19.5" thickBot="1">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="51" t="s">
+        <v>4</v>
+      </c>
+      <c r="O26" s="52"/>
+      <c r="P26" s="52"/>
+      <c r="Q26" s="19">
+        <f>Q25/1000</f>
+        <v>0.8448</v>
+      </c>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+    </row>
+    <row r="38" spans="13:13">
+      <c r="M38" s="39"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S2:S6"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="N26:P26"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O8" r:id="rId1" xr:uid="{CEAFB5A2-1021-46AB-840F-22E9403659CA}"/>
+    <hyperlink ref="O9" r:id="rId2" xr:uid="{0AD504A4-3E61-484E-ACD9-3C0157423F2F}"/>
+    <hyperlink ref="O10" r:id="rId3" xr:uid="{12BB926F-21EB-4860-9790-706509CABA8A}"/>
+    <hyperlink ref="O12" r:id="rId4" xr:uid="{3016A4D6-7174-4FBE-A3DF-C43412AAB1F0}"/>
+    <hyperlink ref="O13" r:id="rId5" xr:uid="{AE7DA16A-30F3-4206-8F14-28F4B94BA671}"/>
+    <hyperlink ref="O15" r:id="rId6" xr:uid="{79A0078A-0988-47E5-9105-2855491EF99F}"/>
+    <hyperlink ref="O16" r:id="rId7" xr:uid="{114A564F-7B1E-4FFC-BA1E-54261E21E17E}"/>
+    <hyperlink ref="O17" r:id="rId8" xr:uid="{EDD6EAEF-6181-48F9-9D5D-8D6E0F5FC51A}"/>
+    <hyperlink ref="O18" r:id="rId9" xr:uid="{5070FBDA-4362-4FDB-8EE9-685281D14265}"/>
+    <hyperlink ref="O19" r:id="rId10" xr:uid="{3E8748E5-2741-4C44-819A-A9B464966821}"/>
+    <hyperlink ref="O20" r:id="rId11" xr:uid="{EED3A9AE-F906-4303-AB8B-E6D64A9D98AF}"/>
+    <hyperlink ref="O21" r:id="rId12" xr:uid="{C1D15EDC-73D2-4B4A-B702-B634361A0F5E}"/>
+    <hyperlink ref="O22" r:id="rId13" xr:uid="{916BFC0C-1094-47B9-AAF9-66FAC6E98601}"/>
+    <hyperlink ref="O23" r:id="rId14" xr:uid="{EE05B829-3A3D-4F87-B1A4-2D1B247DAF7B}"/>
+    <hyperlink ref="O24" r:id="rId15" xr:uid="{7C299554-DCB5-4CCA-81B7-3CF7E884446E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#3 (Added 5 Board Cost Sheet in Main Board)
</commit_message>
<xml_diff>
--- a/Design Files/LLR-05U (Advance Version)/Secondary Board/BOM/eSpark BOM LLR-05U (Secondary-Board).xlsx
+++ b/Design Files/LLR-05U (Advance Version)/Secondary Board/BOM/eSpark BOM LLR-05U (Secondary-Board).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20375"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20409"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\abdullah-liquidlevelrelay\Design Files\LLR-05U (Advance Version)\Secondary Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAE00AFA-0E5E-4294-9649-F4D88036687F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1956B77-BC39-45BE-B7BA-82DC9397E6C4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4965,11 +4965,11 @@
         <v>131</v>
       </c>
       <c r="P24" s="47">
-        <v>1.44E-2</v>
+        <v>2.2200000000000001E-2</v>
       </c>
       <c r="Q24" s="15">
         <f>P24*N24</f>
-        <v>0.28799999999999998</v>
+        <v>0.44400000000000001</v>
       </c>
       <c r="R24" s="14"/>
       <c r="S24" s="20"/>
@@ -4995,7 +4995,7 @@
       <c r="P25" s="52"/>
       <c r="Q25" s="18">
         <f>SUM(Q8:Q24)</f>
-        <v>10.100499999999998</v>
+        <v>10.256499999999999</v>
       </c>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
@@ -5021,7 +5021,7 @@
       <c r="P26" s="52"/>
       <c r="Q26" s="19">
         <f>Q25/5</f>
-        <v>2.0200999999999998</v>
+        <v>2.0512999999999999</v>
       </c>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
@@ -5051,7 +5051,7 @@
     <hyperlink ref="O21" r:id="rId12" xr:uid="{3AA63DEA-B21A-4F9F-8A31-6A3211F1CC8E}"/>
     <hyperlink ref="O22" r:id="rId13" xr:uid="{7E8EEF43-AB22-49DB-8C88-D4CAF04B819B}"/>
     <hyperlink ref="O23" r:id="rId14" xr:uid="{23B72340-7062-40CF-9C96-CF19052BAC73}"/>
-    <hyperlink ref="O24" r:id="rId15" xr:uid="{DBDD888A-19E2-4C45-90AC-B3726FABBC25}"/>
+    <hyperlink ref="O24" r:id="rId15" xr:uid="{6580D18F-B2AB-462A-9C90-D558CDDB22D7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId16"/>
@@ -6164,11 +6164,11 @@
         <v>131</v>
       </c>
       <c r="P24" s="47">
-        <v>1.3899999999999999E-2</v>
+        <v>1.5299999999999999E-2</v>
       </c>
       <c r="Q24" s="15">
         <f>P24*N24</f>
-        <v>13.899999999999999</v>
+        <v>15.299999999999999</v>
       </c>
       <c r="R24" s="14"/>
       <c r="S24" s="20"/>
@@ -6194,7 +6194,7 @@
       <c r="P25" s="52"/>
       <c r="Q25" s="18">
         <f>SUM(Q8:Q24)</f>
-        <v>844.8</v>
+        <v>846.19999999999993</v>
       </c>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
@@ -6220,7 +6220,7 @@
       <c r="P26" s="52"/>
       <c r="Q26" s="19">
         <f>Q25/1000</f>
-        <v>0.8448</v>
+        <v>0.84619999999999995</v>
       </c>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
@@ -6250,7 +6250,7 @@
     <hyperlink ref="O21" r:id="rId12" xr:uid="{C1D15EDC-73D2-4B4A-B702-B634361A0F5E}"/>
     <hyperlink ref="O22" r:id="rId13" xr:uid="{916BFC0C-1094-47B9-AAF9-66FAC6E98601}"/>
     <hyperlink ref="O23" r:id="rId14" xr:uid="{EE05B829-3A3D-4F87-B1A4-2D1B247DAF7B}"/>
-    <hyperlink ref="O24" r:id="rId15" xr:uid="{7C299554-DCB5-4CCA-81B7-3CF7E884446E}"/>
+    <hyperlink ref="O24" r:id="rId15" xr:uid="{B8474985-F7F4-423A-AA8F-7629255B4DAE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId16"/>

</xml_diff>